<commit_message>
Updating files with armazenagem field
</commit_message>
<xml_diff>
--- a/app/media/densidade_concentracao.xlsx
+++ b/app/media/densidade_concentracao.xlsx
@@ -643,7 +643,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>20926963000128</v>
+        <v>20926963000127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1374,7 +1374,7 @@
         <v>13</v>
       </c>
       <c r="E48" s="1" t="n">
-        <v>61133096000312</v>
+        <v>61133096000311</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1408,7 +1408,7 @@
         <v>17</v>
       </c>
       <c r="E50" s="1" t="n">
-        <v>61133096000312</v>
+        <v>61133096000311</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>